<commit_message>
Coconut Grove September: cross-check delinquency tab against September reports, flag Executive Summary row swap
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014HbSR1rcT3CgYHwcF42jpH
</commit_message>
<xml_diff>
--- a/tasks/monthly-reports/outbox/2026-10-16-CGR-september-2026-executive-summary.xlsx
+++ b/tasks/monthly-reports/outbox/2026-10-16-CGR-september-2026-executive-summary.xlsx
@@ -6699,7 +6699,7 @@
       </c>
       <c r="C14" s="300" t="inlineStr">
         <is>
-          <t>Balance reflects September charges. The Third Amendment conditional rent period ended 8/31/2026 and September was the first month back on full Minimum Rent and Additional Rent.</t>
+          <t>Balance reflects September charges. The Third Amendment conditional rent period ended 8/31/2026 and September was the first month back on full Minimum Rent and Additional Rent. No payment received since 6/3/2026.</t>
         </is>
       </c>
       <c r="D14" s="301"/>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="C15" s="300" t="inlineStr">
         <is>
-          <t>Balance reflects September charges ($24,151.97), August CAM ($748.00) and prior year CAM net of credits ($8,563.61). Tenant is negotiating an agreement with Landlord and looking to reopen by November 2026.</t>
+          <t>Balance reflects September charges ($24,151.97), August CAM ($748.00) and prior year CAM and excise tax, net of credits ($8,563.61). Tenant is negotiating an agreement with Landlord and looking to reopen by November 2026.</t>
         </is>
       </c>
       <c r="D15" s="301"/>
@@ -6730,7 +6730,7 @@
       <c r="H15" s="301"/>
       <c r="I15" s="302"/>
     </row>
-    <row r="16" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="91" t="inlineStr">
         <is>
           <t>Laverne's</t>
@@ -6741,7 +6741,7 @@
       </c>
       <c r="C16" s="300" t="inlineStr">
         <is>
-          <t>Balance reflects September charges, including an $880.96 late charge. The Third Amendment conditional rent period ended 8/31/2026 and full rent resumed 9/1/2026.</t>
+          <t>Balance reflects September charges, including an $880.96 late charge. No payment received since 8/13/2026.</t>
         </is>
       </c>
       <c r="D16" s="301"/>

</xml_diff>

<commit_message>
Coconut Grove September delinquency: drop Foster's and Kona Heaven per Emma
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014HbSR1rcT3CgYHwcF42jpH
</commit_message>
<xml_diff>
--- a/tasks/monthly-reports/outbox/2026-10-16-CGR-september-2026-executive-summary.xlsx
+++ b/tasks/monthly-reports/outbox/2026-10-16-CGR-september-2026-executive-summary.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$I$52</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Fosters Rebuild Costs'!$A$1:$E$80</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Tenant COI Tracking '!$A$1:$G$32</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tenant Delinquency'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Tenant Delinquency'!$A$1:$I$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Tenant Maintenance Tracking'!$A$1:$E$28</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -6709,18 +6709,18 @@
       <c r="H14" s="301"/>
       <c r="I14" s="302"/>
     </row>
-    <row r="15" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>Foster's Kitchen</t>
+          <t>Laverne's</t>
         </is>
       </c>
       <c r="B15" s="109">
-        <v>33463.58</v>
+        <v>19330.39</v>
       </c>
       <c r="C15" s="300" t="inlineStr">
         <is>
-          <t>Balance reflects September charges ($24,151.97), August CAM ($748.00) and prior year CAM and excise tax, net of credits ($8,563.61). Tenant is negotiating an agreement with Landlord and looking to reopen by November 2026.</t>
+          <t>Balance reflects September charges, including an $880.96 late charge. No payment received since 8/13/2026.</t>
         </is>
       </c>
       <c r="D15" s="301"/>
@@ -6730,18 +6730,18 @@
       <c r="H15" s="301"/>
       <c r="I15" s="302"/>
     </row>
-    <row r="16" spans="1:16" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="91" t="inlineStr">
         <is>
-          <t>Laverne's</t>
+          <t>Lucasie</t>
         </is>
       </c>
       <c r="B16" s="109">
-        <v>19330.39</v>
+        <v>14659.08</v>
       </c>
       <c r="C16" s="300" t="inlineStr">
         <is>
-          <t>Balance reflects September charges, including an $880.96 late charge. No payment received since 8/13/2026.</t>
+          <t>Balance reflects September charges ($11,538.95, including a $525.87 late charge) plus $3,120.13 from 2026 NNN short pays and 2025 PYC, offset by 2024 PYC credit. Working with Nir Levav to pay the remaining balance.</t>
         </is>
       </c>
       <c r="D16" s="301"/>
@@ -6751,74 +6751,32 @@
       <c r="H16" s="301"/>
       <c r="I16" s="302"/>
     </row>
-    <row r="17" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="91" t="inlineStr">
-        <is>
-          <t>Lucasie</t>
-        </is>
-      </c>
-      <c r="B17" s="109">
-        <v>14659.08</v>
-      </c>
-      <c r="C17" s="300" t="inlineStr">
-        <is>
-          <t>Balance reflects September charges ($11,538.95, including a $525.87 late charge) plus $3,120.13 from 2026 NNN short pays and 2025 PYC, offset by 2024 PYC credit. Working with Nir Levav to pay the remaining balance.</t>
-        </is>
-      </c>
-      <c r="D17" s="301"/>
-      <c r="E17" s="301"/>
-      <c r="F17" s="301"/>
-      <c r="G17" s="301"/>
-      <c r="H17" s="301"/>
-      <c r="I17" s="302"/>
-    </row>
-    <row r="18" spans="1:16" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="91" t="inlineStr">
-        <is>
-          <t>Kona Heaven Coffee (Café Kona)</t>
-        </is>
-      </c>
-      <c r="B18" s="109">
-        <v>6958.31</v>
-      </c>
-      <c r="C18" s="300" t="inlineStr">
-        <is>
-          <t>Balance reflects the 2024 PYC billed 5/1/2025. Landlord approved waiving it as part of the renewal and Management will clear it internally.</t>
-        </is>
-      </c>
-      <c r="D18" s="301"/>
-      <c r="E18" s="301"/>
-      <c r="F18" s="301"/>
-      <c r="G18" s="301"/>
-      <c r="H18" s="301"/>
-      <c r="I18" s="302"/>
-    </row>
-    <row r="19" spans="1:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="88" t="s">
+    <row r="17" spans="1:16" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="88" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="89">
-        <f>SUM(B13:B18)</f>
-        <v>190400.88</v>
-      </c>
-      <c r="C19" s="93"/>
-      <c r="D19" s="93"/>
-      <c r="E19" s="93"/>
-      <c r="F19" s="93"/>
-      <c r="G19" s="93"/>
-      <c r="H19" s="93"/>
-      <c r="I19" s="94"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="58"/>
-      <c r="B20" s="59"/>
-      <c r="C20" s="58"/>
-      <c r="D20" s="58"/>
-      <c r="E20" s="58"/>
-      <c r="F20" s="58"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="58"/>
-      <c r="I20" s="1"/>
+      <c r="B17" s="89">
+        <f>SUM(B13:B16)</f>
+        <v>149978.99</v>
+      </c>
+      <c r="C17" s="93"/>
+      <c r="D17" s="93"/>
+      <c r="E17" s="93"/>
+      <c r="F17" s="93"/>
+      <c r="G17" s="93"/>
+      <c r="H17" s="93"/>
+      <c r="I17" s="94"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="58"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="58"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58"/>
+      <c r="H18" s="58"/>
+      <c r="I18" s="1"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="100"/>
@@ -6858,7 +6816,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="10">
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="C12:I12"/>
@@ -6869,8 +6827,6 @@
     <mergeCell ref="C14:I14"/>
     <mergeCell ref="C15:I15"/>
     <mergeCell ref="C16:I16"/>
-    <mergeCell ref="C17:I17"/>
-    <mergeCell ref="C18:I18"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>